<commit_message>
Updated data for STP
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/dynamic_field.xlsx
+++ b/mosip_master/xlsx/dynamic_field.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\eclipse-workspace\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3958B1B7-913A-430F-A169-A703770CF1DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9FC4F5-47A5-4FB6-A06F-356858ACB543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$41</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="68">
   <si>
     <t>id</t>
   </si>
@@ -348,6 +348,47 @@
 		"code": "DI",
 		"value": "Deplacé interne"
 	}</t>
+  </si>
+  <si>
+    <t>passportIssuingCountry</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>countryOfCitizenship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+{
+	"code": "ST",
+	"value": "São Tomé and Príncipe"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+{
+	"code": "IN",
+	"value": "India"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+{
+	"code": "US",
+	"value": "United States"
+}
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+{
+	"code": "US",
+	"value": "United States"
+}</t>
   </si>
 </sst>
 </file>
@@ -404,7 +445,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -429,11 +470,42 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -730,12 +802,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.54296875" style="6" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="17.6328125" customWidth="1"/>
+    <col min="3" max="3" width="26.26953125" customWidth="1"/>
     <col min="4" max="4" width="21.54296875" customWidth="1"/>
     <col min="5" max="5" width="32.54296875" customWidth="1"/>
     <col min="6" max="6" width="15.6328125" bestFit="1" customWidth="1"/>
@@ -1254,7 +1326,7 @@
         <v>40</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G18" s="8" t="b">
         <v>1</v>
@@ -1268,7 +1340,7 @@
     </row>
     <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>10313</v>
+        <v>10312</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>38</v>
@@ -1280,97 +1352,97 @@
         <v>9</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="5">
+        <v>10313</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G19" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="6">
-        <v>10314</v>
-      </c>
-      <c r="B20" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F20" t="s">
-        <v>41</v>
-      </c>
-      <c r="G20" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="6">
-        <v>10315</v>
-      </c>
-      <c r="B21" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="G20" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>10311</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F21" t="s">
-        <v>41</v>
-      </c>
-      <c r="G21" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" t="s">
-        <v>11</v>
-      </c>
-      <c r="I21" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A22" s="6">
-        <v>10188</v>
+        <v>10314</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C22" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D22" t="s">
         <v>9</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="F22" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G22" s="9" t="b">
         <v>1</v>
@@ -1384,22 +1456,22 @@
     </row>
     <row r="23" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A23" s="6">
-        <v>10016</v>
+        <v>10315</v>
       </c>
       <c r="B23" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C23" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D23" t="s">
         <v>9</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="F23" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G23" s="9" t="b">
         <v>1</v>
@@ -1413,7 +1485,7 @@
     </row>
     <row r="24" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A24" s="6">
-        <v>10017</v>
+        <v>10188</v>
       </c>
       <c r="B24" t="s">
         <v>13</v>
@@ -1425,7 +1497,7 @@
         <v>9</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="F24" t="s">
         <v>10</v>
@@ -1442,7 +1514,7 @@
     </row>
     <row r="25" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A25" s="6">
-        <v>10018</v>
+        <v>10016</v>
       </c>
       <c r="B25" t="s">
         <v>13</v>
@@ -1454,7 +1526,7 @@
         <v>9</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="F25" t="s">
         <v>10</v>
@@ -1471,7 +1543,7 @@
     </row>
     <row r="26" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A26" s="6">
-        <v>10019</v>
+        <v>10017</v>
       </c>
       <c r="B26" t="s">
         <v>13</v>
@@ -1483,10 +1555,10 @@
         <v>9</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F26" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="G26" s="9" t="b">
         <v>1</v>
@@ -1500,7 +1572,7 @@
     </row>
     <row r="27" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A27" s="6">
-        <v>10020</v>
+        <v>10018</v>
       </c>
       <c r="B27" t="s">
         <v>13</v>
@@ -1512,10 +1584,10 @@
         <v>9</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F27" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="G27" s="9" t="b">
         <v>1</v>
@@ -1529,7 +1601,7 @@
     </row>
     <row r="28" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A28" s="6">
-        <v>10021</v>
+        <v>10019</v>
       </c>
       <c r="B28" t="s">
         <v>13</v>
@@ -1541,7 +1613,7 @@
         <v>9</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F28" t="s">
         <v>41</v>
@@ -1558,7 +1630,7 @@
     </row>
     <row r="29" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A29" s="6">
-        <v>10022</v>
+        <v>10020</v>
       </c>
       <c r="B29" t="s">
         <v>13</v>
@@ -1570,7 +1642,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F29" t="s">
         <v>41</v>
@@ -1587,19 +1659,19 @@
     </row>
     <row r="30" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A30" s="6">
-        <v>10023</v>
+        <v>10021</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C30" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F30" t="s">
         <v>41</v>
@@ -1616,19 +1688,19 @@
     </row>
     <row r="31" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A31" s="6">
-        <v>10024</v>
+        <v>10022</v>
       </c>
       <c r="B31" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C31" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="D31" t="s">
         <v>9</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F31" t="s">
         <v>41</v>
@@ -1645,7 +1717,7 @@
     </row>
     <row r="32" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A32" s="6">
-        <v>10025</v>
+        <v>10023</v>
       </c>
       <c r="B32" t="s">
         <v>35</v>
@@ -1657,7 +1729,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F32" t="s">
         <v>41</v>
@@ -1672,9 +1744,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A33" s="6">
-        <v>10026</v>
+        <v>10024</v>
       </c>
       <c r="B33" t="s">
         <v>35</v>
@@ -1686,7 +1758,7 @@
         <v>9</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F33" t="s">
         <v>41</v>
@@ -1701,9 +1773,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A34" s="6">
-        <v>10089</v>
+        <v>10025</v>
       </c>
       <c r="B34" t="s">
         <v>35</v>
@@ -1715,7 +1787,7 @@
         <v>9</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F34" t="s">
         <v>41</v>
@@ -1730,9 +1802,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A35" s="6">
-        <v>10090</v>
+        <v>10026</v>
       </c>
       <c r="B35" t="s">
         <v>35</v>
@@ -1744,10 +1816,10 @@
         <v>9</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F35" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G35" s="9" t="b">
         <v>1</v>
@@ -1759,9 +1831,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A36" s="6">
-        <v>10091</v>
+        <v>10089</v>
       </c>
       <c r="B36" t="s">
         <v>35</v>
@@ -1773,10 +1845,10 @@
         <v>9</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F36" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G36" s="9" t="b">
         <v>1</v>
@@ -1788,9 +1860,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A37" s="6">
-        <v>10011</v>
+        <v>10090</v>
       </c>
       <c r="B37" t="s">
         <v>35</v>
@@ -1802,7 +1874,7 @@
         <v>9</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F37" t="s">
         <v>10</v>
@@ -1817,9 +1889,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A38" s="6">
-        <v>10123</v>
+        <v>10091</v>
       </c>
       <c r="B38" t="s">
         <v>35</v>
@@ -1831,7 +1903,7 @@
         <v>9</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F38" t="s">
         <v>10</v>
@@ -1846,9 +1918,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A39" s="6">
-        <v>10094</v>
+        <v>10011</v>
       </c>
       <c r="B39" t="s">
         <v>35</v>
@@ -1860,28 +1932,449 @@
         <v>9</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F39" t="s">
+        <v>10</v>
+      </c>
+      <c r="G39" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H39" t="s">
+        <v>11</v>
+      </c>
+      <c r="I39" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="6">
+        <v>10123</v>
+      </c>
+      <c r="B40" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F40" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H40" t="s">
+        <v>11</v>
+      </c>
+      <c r="I40" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="6">
+        <v>10094</v>
+      </c>
+      <c r="B41" t="s">
+        <v>35</v>
+      </c>
+      <c r="C41" t="s">
+        <v>35</v>
+      </c>
+      <c r="D41" t="s">
+        <v>9</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F39" t="s">
-        <v>10</v>
-      </c>
-      <c r="G39" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H39" t="s">
-        <v>11</v>
-      </c>
-      <c r="I39" t="s">
-        <v>12</v>
-      </c>
+      <c r="F41" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H41" t="s">
+        <v>11</v>
+      </c>
+      <c r="I41" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="6">
+        <v>12001</v>
+      </c>
+      <c r="B42" t="s">
+        <v>60</v>
+      </c>
+      <c r="C42" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F42" t="s">
+        <v>10</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H42" t="s">
+        <v>62</v>
+      </c>
+      <c r="I42" t="s">
+        <v>12</v>
+      </c>
+      <c r="K42" s="10"/>
+    </row>
+    <row r="43" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A43" s="6">
+        <v>12002</v>
+      </c>
+      <c r="B43" t="s">
+        <v>60</v>
+      </c>
+      <c r="C43" t="s">
+        <v>60</v>
+      </c>
+      <c r="D43" t="s">
+        <v>9</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F43" t="s">
+        <v>41</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H43" t="s">
+        <v>62</v>
+      </c>
+      <c r="I43" t="s">
+        <v>12</v>
+      </c>
+      <c r="K43" s="10"/>
+    </row>
+    <row r="44" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A44" s="6">
+        <v>12003</v>
+      </c>
+      <c r="B44" t="s">
+        <v>60</v>
+      </c>
+      <c r="C44" t="s">
+        <v>60</v>
+      </c>
+      <c r="D44" t="s">
+        <v>9</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F44" t="s">
+        <v>10</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H44" t="s">
+        <v>62</v>
+      </c>
+      <c r="I44" t="s">
+        <v>12</v>
+      </c>
+      <c r="K44" s="10"/>
+    </row>
+    <row r="45" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="6">
+        <v>12004</v>
+      </c>
+      <c r="B45" t="s">
+        <v>60</v>
+      </c>
+      <c r="C45" t="s">
+        <v>60</v>
+      </c>
+      <c r="D45" t="s">
+        <v>9</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F45" t="s">
+        <v>41</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H45" t="s">
+        <v>62</v>
+      </c>
+      <c r="I45" t="s">
+        <v>12</v>
+      </c>
+      <c r="K45" s="10"/>
+    </row>
+    <row r="46" spans="1:11" ht="87" x14ac:dyDescent="0.35">
+      <c r="A46" s="6">
+        <v>12005</v>
+      </c>
+      <c r="B46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C46" t="s">
+        <v>60</v>
+      </c>
+      <c r="D46" t="s">
+        <v>9</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H46" t="s">
+        <v>62</v>
+      </c>
+      <c r="I46" t="s">
+        <v>12</v>
+      </c>
+      <c r="K46" s="10"/>
+    </row>
+    <row r="47" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A47" s="6">
+        <v>12006</v>
+      </c>
+      <c r="B47" t="s">
+        <v>60</v>
+      </c>
+      <c r="C47" t="s">
+        <v>60</v>
+      </c>
+      <c r="D47" t="s">
+        <v>9</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F47" t="s">
+        <v>41</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H47" t="s">
+        <v>62</v>
+      </c>
+      <c r="I47" t="s">
+        <v>12</v>
+      </c>
+      <c r="K47" s="10"/>
+    </row>
+    <row r="48" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A48" s="6">
+        <v>11001</v>
+      </c>
+      <c r="B48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" t="s">
+        <v>63</v>
+      </c>
+      <c r="D48" t="s">
+        <v>9</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F48" t="s">
+        <v>10</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H48" t="s">
+        <v>62</v>
+      </c>
+      <c r="I48" t="s">
+        <v>12</v>
+      </c>
+      <c r="K48" s="10"/>
+    </row>
+    <row r="49" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A49" s="6">
+        <v>11002</v>
+      </c>
+      <c r="B49" t="s">
+        <v>63</v>
+      </c>
+      <c r="C49" t="s">
+        <v>63</v>
+      </c>
+      <c r="D49" t="s">
+        <v>9</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F49" t="s">
+        <v>41</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H49" t="s">
+        <v>62</v>
+      </c>
+      <c r="I49" t="s">
+        <v>12</v>
+      </c>
+      <c r="K49" s="10"/>
+    </row>
+    <row r="50" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A50" s="6">
+        <v>11003</v>
+      </c>
+      <c r="B50" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50" t="s">
+        <v>63</v>
+      </c>
+      <c r="D50" t="s">
+        <v>9</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F50" t="s">
+        <v>10</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H50" t="s">
+        <v>62</v>
+      </c>
+      <c r="I50" t="s">
+        <v>12</v>
+      </c>
+      <c r="K50" s="10"/>
+    </row>
+    <row r="51" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A51" s="6">
+        <v>11004</v>
+      </c>
+      <c r="B51" t="s">
+        <v>63</v>
+      </c>
+      <c r="C51" t="s">
+        <v>63</v>
+      </c>
+      <c r="D51" t="s">
+        <v>9</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F51" t="s">
+        <v>41</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H51" t="s">
+        <v>62</v>
+      </c>
+      <c r="I51" t="s">
+        <v>12</v>
+      </c>
+      <c r="K51" s="10"/>
+    </row>
+    <row r="52" spans="1:11" ht="87" x14ac:dyDescent="0.35">
+      <c r="A52" s="6">
+        <v>11005</v>
+      </c>
+      <c r="B52" t="s">
+        <v>63</v>
+      </c>
+      <c r="C52" t="s">
+        <v>63</v>
+      </c>
+      <c r="D52" t="s">
+        <v>9</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F52" t="s">
+        <v>10</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H52" t="s">
+        <v>62</v>
+      </c>
+      <c r="I52" t="s">
+        <v>12</v>
+      </c>
+      <c r="K52" s="10"/>
+    </row>
+    <row r="53" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A53" s="6">
+        <v>11006</v>
+      </c>
+      <c r="B53" t="s">
+        <v>63</v>
+      </c>
+      <c r="C53" t="s">
+        <v>63</v>
+      </c>
+      <c r="D53" t="s">
+        <v>9</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F53" t="s">
+        <v>41</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H53" t="s">
+        <v>62</v>
+      </c>
+      <c r="I53" t="s">
+        <v>12</v>
+      </c>
+      <c r="K53" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I39" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I41" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A14:A39">
-    <cfRule type="duplicateValues" dxfId="0" priority="10"/>
+  <conditionalFormatting sqref="A14:A41">
+    <cfRule type="duplicateValues" dxfId="3" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>